<commit_message>
feat: release time slot on completed bookings and prevent simultaneous booking conflicts
</commit_message>
<xml_diff>
--- a/Photodate_Test_Cases_Checklist.xlsx
+++ b/Photodate_Test_Cases_Checklist.xlsx
@@ -545,7 +545,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J72"/>
   <cols>
     <col min="1" max="1" width="15.83203125" customWidth="1"/>
     <col min="2" max="2" width="28.83203125" customWidth="1"/>
@@ -566,7 +566,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tổng cộng: 66 Test Cases | Đầy đủ 12 Phân hệ chức năng</v>
+        <v>Tổng cộng: 68 Test Cases | Đầy đủ 12 Phân hệ chức năng</v>
       </c>
     </row>
     <row r="4">
@@ -1322,632 +1322,700 @@
     </row>
     <row r="26" xml:space="preserve">
       <c r="A26" t="str">
+        <v>TC_BOOK_008</v>
+      </c>
+      <c r="B26" t="str">
+        <v>3. Đặt Lịch Chụp Ảnh (Booking)</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Ngăn chặn trùng lịch khi 2 khách đặt cùng lúc (Concurrency Safety)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>NAG đã có 1 đơn chốt (confirmed) trong khung giờ X ngày Y</v>
+      </c>
+      <c r="E26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Khách thứ hai chọn cùng NAG, cùng ngày Y và khung giờ X
+2. Bấm Gửi yêu cầu đặt lịch (trên BookingPage hoặc BookingModal)
+3. Quan sát phản hồi từ hệ thống</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Hệ thống tự động phát hiện xung đột thời gian thực, từ chối tạo đơn trùng (HTTP 409 Conflict), thông báo rõ ràng cho khách chọn khung giờ khác.</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I26" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J26" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="27" xml:space="preserve">
+      <c r="A27" t="str">
+        <v>TC_BOOK_009</v>
+      </c>
+      <c r="B27" t="str">
+        <v>3. Đặt Lịch Chụp Ảnh (Booking)</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Giải phóng thời gian trống khi NAG bấm "Đã Chụp Xong" hoặc "Đã Hủy"</v>
+      </c>
+      <c r="D27" t="str">
+        <v>NAG có 1 đơn lịch đang ở trạng thái confirmed (đang khóa slot)</v>
+      </c>
+      <c r="E27" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. NAG vào Studio Workspace -&gt; Tab Lịch Booking -&gt; Bấm [Đã Chụp Xong] (completed)
+2. Một khách hàng mới vào đặt lịch đúng khung giờ đó của ngày đó
+3. Quan sát hệ thống kiểm tra tình trạng bận/rảnh</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Khung giờ đó được tự động giải phóng (bỏ thời gian trống ra), không còn bị báo bận, khách mới có thể đặt lịch bình thường.</v>
+      </c>
+      <c r="G27" t="str">
+        <v>High</v>
+      </c>
+      <c r="H27" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I27" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J27" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="28" xml:space="preserve">
+      <c r="A28" t="str">
         <v>TC_PHOTO_001</v>
       </c>
-      <c r="B26" t="str">
+      <c r="B28" t="str">
         <v>4. Hồ Sơ Nhiếp Ảnh Gia</v>
       </c>
-      <c r="C26" t="str">
+      <c r="C28" t="str">
         <v>Xem danh sách Nhiếp ảnh gia tại trang /photographers</v>
       </c>
-      <c r="D26" t="str">
+      <c r="D28" t="str">
         <v>Truy cập /photographers</v>
       </c>
-      <c r="E26" t="str" xml:space="preserve">
+      <c r="E28" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Xem lưới danh sách các Nhiếp ảnh gia đối tác
 2. Kiểm tra thông tin hiển thị trên từng thẻ</v>
       </c>
-      <c r="F26" t="str">
+      <c r="F28" t="str">
         <v>Mỗi thẻ hiển thị: Avatar/Logo, Tên NAG, Khu vực hoạt động, Thể loại sở trường, Số album đã thực hiện, Đánh giá sao, Link xem hồ sơ.</v>
       </c>
-      <c r="G26" t="str">
-        <v>High</v>
-      </c>
-      <c r="H26" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I26" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J26" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="27" xml:space="preserve">
-      <c r="A27" t="str">
+      <c r="G28" t="str">
+        <v>High</v>
+      </c>
+      <c r="H28" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I28" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J28" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="29" xml:space="preserve">
+      <c r="A29" t="str">
         <v>TC_PHOTO_002</v>
       </c>
-      <c r="B27" t="str">
+      <c r="B29" t="str">
         <v>4. Hồ Sơ Nhiếp Ảnh Gia</v>
       </c>
-      <c r="C27" t="str">
+      <c r="C29" t="str">
         <v>Tìm kiếm thợ ảnh theo Tên, Email, Thiết bị, Tỉnh thành</v>
       </c>
-      <c r="D27" t="str">
+      <c r="D29" t="str">
         <v>Ở trang /photographers</v>
       </c>
-      <c r="E27" t="str" xml:space="preserve">
+      <c r="E29" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Gõ từ khóa tìm kiếm (VD: "Sony", "Hà Nội", "Cưới") vào ô tìm kiếm
 2. Quan sát kết quả lọc</v>
       </c>
-      <c r="F27" t="str">
+      <c r="F29" t="str">
         <v>Danh sách lọc tức thời theo thời gian thực (Real-time filtering), khớp chính xác với tiêu chí.</v>
       </c>
-      <c r="G27" t="str">
-        <v>High</v>
-      </c>
-      <c r="H27" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I27" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J27" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="28" xml:space="preserve">
-      <c r="A28" t="str">
+      <c r="G29" t="str">
+        <v>High</v>
+      </c>
+      <c r="H29" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I29" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J29" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="30" xml:space="preserve">
+      <c r="A30" t="str">
         <v>TC_PHOTO_003</v>
       </c>
-      <c r="B28" t="str">
+      <c r="B30" t="str">
         <v>4. Hồ Sơ Nhiếp Ảnh Gia</v>
       </c>
-      <c r="C28" t="str">
+      <c r="C30" t="str">
         <v>Xem Trang Hồ Sơ Chi Tiết Nhiếp Ảnh Gia (/photographer/:id)</v>
       </c>
-      <c r="D28" t="str">
+      <c r="D30" t="str">
         <v>Bấm vào 1 Nhiếp ảnh gia cụ thể</v>
       </c>
-      <c r="E28" t="str" xml:space="preserve">
+      <c r="E30" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Quan sát phần Header: Cover, Avatar, Tên Studio, Đánh giá
 2. Xem tab "Giới Thiệu": Bio năng lực, Thiết bị chính, Kinh nghiệm, Địa chỉ Studio
 3. Xem tab "Bộ Sưu Tập": Các album ảnh mẫu đã đăng tải
 4. Xem tab "Đánh Giá": Nhận xét của khách hàng</v>
       </c>
-      <c r="F28" t="str">
+      <c r="F30" t="str">
         <v>Hiển thị chuyên nghiệp, đẳng cấp, đầy đủ các thông số năng lực thực tế.</v>
       </c>
-      <c r="G28" t="str">
-        <v>High</v>
-      </c>
-      <c r="H28" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I28" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J28" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="29" xml:space="preserve">
-      <c r="A29" t="str">
+      <c r="G30" t="str">
+        <v>High</v>
+      </c>
+      <c r="H30" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I30" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J30" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="31" xml:space="preserve">
+      <c r="A31" t="str">
         <v>TC_PHOTO_004</v>
       </c>
-      <c r="B29" t="str">
+      <c r="B31" t="str">
         <v>4. Hồ Sơ Nhiếp Ảnh Gia</v>
       </c>
-      <c r="C29" t="str">
+      <c r="C31" t="str">
         <v>Liên hệ nhanh qua Zalo &amp; Gọi Hotline của Nhiếp ảnh gia</v>
       </c>
-      <c r="D29" t="str">
+      <c r="D31" t="str">
         <v>Đang ở trang chi tiết NAG</v>
       </c>
-      <c r="E29" t="str" xml:space="preserve">
+      <c r="E31" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút "Chat Zalo"
 2. Bấm nút "Gọi Điện / Hotline"</v>
       </c>
-      <c r="F29" t="str">
+      <c r="F31" t="str">
         <v>Nút Zalo mở link zalo.me chính xác theo số điện thoại NAG; nút Gọi mở ứng dụng gọi điện trên thiết bị.</v>
       </c>
-      <c r="G29" t="str">
+      <c r="G31" t="str">
         <v>Medium</v>
       </c>
-      <c r="H29" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I29" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J29" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="30" xml:space="preserve">
-      <c r="A30" t="str">
+      <c r="H31" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I31" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J31" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="32" xml:space="preserve">
+      <c r="A32" t="str">
         <v>TC_PHOTO_005</v>
       </c>
-      <c r="B30" t="str">
+      <c r="B32" t="str">
         <v>4. Hồ Sơ Nhiếp Ảnh Gia</v>
       </c>
-      <c r="C30" t="str">
+      <c r="C32" t="str">
         <v>Đặt lịch chụp chỉ định trực tiếp từ trang cá nhân NAG</v>
       </c>
-      <c r="D30" t="str">
+      <c r="D32" t="str">
         <v>Đang ở trang chi tiết NAG</v>
       </c>
-      <c r="E30" t="str" xml:space="preserve">
+      <c r="E32" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút "Đặt Lịch Chụp Ngay Với [Tên NAG]"
 2. Kiểm tra form Đặt lịch mở ra</v>
       </c>
-      <c r="F30" t="str">
+      <c r="F32" t="str">
         <v>Form đặt lịch mở lên với trường Nhiếp ảnh gia và Tỉnh thành đã được chọn cố định theo đúng NAG đó.</v>
       </c>
-      <c r="G30" t="str">
-        <v>High</v>
-      </c>
-      <c r="H30" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I30" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J30" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="31" xml:space="preserve">
-      <c r="A31" t="str">
+      <c r="G32" t="str">
+        <v>High</v>
+      </c>
+      <c r="H32" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I32" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J32" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="33" xml:space="preserve">
+      <c r="A33" t="str">
         <v>TC_STUDIO_001</v>
       </c>
-      <c r="B31" t="str">
+      <c r="B33" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C31" t="str">
+      <c r="C33" t="str">
         <v>Cài đặt Studio &amp; Hồ sơ năng lực trong Workspace</v>
       </c>
-      <c r="D31" t="str">
+      <c r="D33" t="str">
         <v>Đăng nhập tài khoản NAG -&gt; Truy cập /app</v>
       </c>
-      <c r="E31" t="str" xml:space="preserve">
+      <c r="E33" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Vào mục "Cài Đặt Studio &amp; Hồ Sơ"
 2. Cập nhật Tỉnh/Thành, Phường/Xã Studio, Địa chỉ số nhà
 3. Cập nhật Bio, Thiết bị máy ảnh, Giá khởi điểm, Phong cách chụp
 4. Bấm "Lưu Cấu Hình"</v>
       </c>
-      <c r="F31" t="str">
+      <c r="F33" t="str">
         <v>Hệ thống thông báo cập nhật thành công, dữ liệu được đồng bộ ngay lên trang công khai của NAG.</v>
       </c>
-      <c r="G31" t="str">
-        <v>High</v>
-      </c>
-      <c r="H31" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I31" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J31" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="32" xml:space="preserve">
-      <c r="A32" t="str">
+      <c r="G33" t="str">
+        <v>High</v>
+      </c>
+      <c r="H33" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I33" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J33" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="34" xml:space="preserve">
+      <c r="A34" t="str">
         <v>TC_STUDIO_002</v>
       </c>
-      <c r="B32" t="str">
+      <c r="B34" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C32" t="str">
+      <c r="C34" t="str">
         <v>Tạo Album ảnh mới &amp; Thiết lập mã PIN bảo mật</v>
       </c>
-      <c r="D32" t="str">
+      <c r="D34" t="str">
         <v>Ở trang Studio Workspace -&gt; Quản lý Album</v>
       </c>
-      <c r="E32" t="str" xml:space="preserve">
+      <c r="E34" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút "Tạo Album Mới"
 2. Nhập Tên Album (VD: Kỷ Yếu Lớp 12A1), Tên Khách hàng, SĐT
 3. Nhập Mã PIN bảo mật (4-6 số)
 4. Đặt Hạn mức số ảnh chọn (VD: Tối đa 35 ảnh)
 5. Bấm "Khởi Tạo Album"</v>
       </c>
-      <c r="F32" t="str">
+      <c r="F34" t="str">
         <v>Album được tạo thành công, xuất hiện trong danh sách album đang quản lý của Studio.</v>
       </c>
-      <c r="G32" t="str">
-        <v>High</v>
-      </c>
-      <c r="H32" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I32" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J32" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="33" xml:space="preserve">
-      <c r="A33" t="str">
+      <c r="G34" t="str">
+        <v>High</v>
+      </c>
+      <c r="H34" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I34" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J34" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="35" xml:space="preserve">
+      <c r="A35" t="str">
         <v>TC_STUDIO_003</v>
       </c>
-      <c r="B33" t="str">
+      <c r="B35" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C33" t="str">
+      <c r="C35" t="str">
         <v>Tải ảnh hàng loạt lên Album (Bulk Photo Upload)</v>
       </c>
-      <c r="D33" t="str">
+      <c r="D35" t="str">
         <v>Album vừa tạo đang mở</v>
       </c>
-      <c r="E33" t="str" xml:space="preserve">
+      <c r="E35" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Kéo thả 20-50 bức ảnh chất lượng cao vào khu vực upload
 2. Theo dõi tiến trình tải lên (Upload Progress Bar)
 3. Quan sát các ảnh xuất hiện trên lưới sau khi tải xong</v>
       </c>
-      <c r="F33" t="str">
+      <c r="F35" t="str">
         <v>Tải lên hoàn tất, ảnh hiển thị sắc nét, giữ nguyên tỷ lệ và chất lượng hình ảnh gốc.</v>
       </c>
-      <c r="G33" t="str">
-        <v>High</v>
-      </c>
-      <c r="H33" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I33" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J33" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="34" xml:space="preserve">
-      <c r="A34" t="str">
+      <c r="G35" t="str">
+        <v>High</v>
+      </c>
+      <c r="H35" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I35" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J35" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="36" xml:space="preserve">
+      <c r="A36" t="str">
         <v>TC_STUDIO_004</v>
       </c>
-      <c r="B34" t="str">
+      <c r="B36" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C34" t="str">
+      <c r="C36" t="str">
         <v>Cấu hình Watermark (Đóng dấu ảnh xem trước chống trộm ảnh)</v>
       </c>
-      <c r="D34" t="str">
+      <c r="D36" t="str">
         <v>Ở phần cài đặt album</v>
       </c>
-      <c r="E34" t="str" xml:space="preserve">
+      <c r="E36" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bật tính năng "Đóng dấu Watermark"
 2. Nhập chữ đóng dấu (VD: "Studio Poseidon") hoặc tải logo mờ
 3. Chọn vị trí đóng dấu (Chính giữa / Góc dưới)
 4. Bấm Lưu</v>
       </c>
-      <c r="F34" t="str">
+      <c r="F36" t="str">
         <v>Ảnh xem trước của khách hàng tự động được chèn watermark mờ chống sao chép bản quyền.</v>
       </c>
-      <c r="G34" t="str">
+      <c r="G36" t="str">
         <v>Medium</v>
       </c>
-      <c r="H34" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I34" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J34" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="35" xml:space="preserve">
-      <c r="A35" t="str">
+      <c r="H36" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I36" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J36" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="37" xml:space="preserve">
+      <c r="A37" t="str">
         <v>TC_STUDIO_005</v>
       </c>
-      <c r="B35" t="str">
+      <c r="B37" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C35" t="str">
+      <c r="C37" t="str">
         <v>Sao chép Link chia sẻ Album &amp; Mã PIN gửi cho khách hàng</v>
       </c>
-      <c r="D35" t="str">
+      <c r="D37" t="str">
         <v>Album đã có ảnh</v>
       </c>
-      <c r="E35" t="str" xml:space="preserve">
+      <c r="E37" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Tại thẻ album, bấm "Sao chép Link Album"
 2. Bấm "Sao chép Tin nhắn bàn giao (kèm mã PIN)"
 3. Dán ra ghi chú kiểm tra định dạng tin nhắn</v>
       </c>
-      <c r="F35" t="str">
+      <c r="F37" t="str">
         <v>Tin nhắn mẫu soạn sẵn link album dạng https://.../album/:id và mã PIN tiện lợi cho khách hàng.</v>
       </c>
-      <c r="G35" t="str">
-        <v>High</v>
-      </c>
-      <c r="H35" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I35" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J35" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="36" xml:space="preserve">
-      <c r="A36" t="str">
+      <c r="G37" t="str">
+        <v>High</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I37" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J37" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="38" xml:space="preserve">
+      <c r="A38" t="str">
         <v>TC_STUDIO_006</v>
       </c>
-      <c r="B36" t="str">
+      <c r="B38" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C36" t="str">
+      <c r="C38" t="str">
         <v>Theo dõi tiến độ khách hàng chọn ảnh (Selection Status)</v>
       </c>
-      <c r="D36" t="str">
+      <c r="D38" t="str">
         <v>Khách hàng đã tiến hành chọn ảnh</v>
       </c>
-      <c r="E36" t="str" xml:space="preserve">
+      <c r="E38" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Xem thẻ album trong Workspace
 2. Kiểm tra thanh trạng thái: Khách đang chọn / Khách đã gửi danh sách
 3. Xem số lượng ảnh khách đã duyệt</v>
       </c>
-      <c r="F36" t="str">
+      <c r="F38" t="str">
         <v>Trạng thái cập nhật theo thời gian thực, hiển thị danh sách các bức ảnh khách yêu thích kèm ghi chú.</v>
       </c>
-      <c r="G36" t="str">
-        <v>High</v>
-      </c>
-      <c r="H36" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I36" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J36" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="37" xml:space="preserve">
-      <c r="A37" t="str">
+      <c r="G38" t="str">
+        <v>High</v>
+      </c>
+      <c r="H38" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I38" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J38" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="39" xml:space="preserve">
+      <c r="A39" t="str">
         <v>TC_STUDIO_007</v>
       </c>
-      <c r="B37" t="str">
+      <c r="B39" t="str">
         <v>5. Studio Workspace (Cho NAG)</v>
       </c>
-      <c r="C37" t="str">
+      <c r="C39" t="str">
         <v>Quản lý Đơn đặt lịch gửi đến Studio (Bookings CRM)</v>
       </c>
-      <c r="D37" t="str">
+      <c r="D39" t="str">
         <v>Có khách hàng đặt lịch với NAG này</v>
       </c>
-      <c r="E37" t="str" xml:space="preserve">
+      <c r="E39" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Vào mục "Lịch Chụp Đã Nhận"
 2. Xem chi tiết đơn đặt lịch: Tên khách, SĐT, Gói chụp, Ngày giờ, Địa điểm
 3. Thao tác: Bấm "Xác Nhận Nhận Lịch" hoặc "Từ Chối"</v>
       </c>
-      <c r="F37" t="str">
+      <c r="F39" t="str">
         <v>Cập nhật trạng thái đơn chụp, khách hàng tra cứu sẽ thấy trạng thái đã được xác nhận.</v>
       </c>
-      <c r="G37" t="str">
-        <v>High</v>
-      </c>
-      <c r="H37" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I37" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J37" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="38" xml:space="preserve">
-      <c r="A38" t="str">
+      <c r="G39" t="str">
+        <v>High</v>
+      </c>
+      <c r="H39" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I39" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J39" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="40" xml:space="preserve">
+      <c r="A40" t="str">
         <v>TC_CLIENT_001</v>
       </c>
-      <c r="B38" t="str">
+      <c r="B40" t="str">
         <v>6. Khách Hàng Xem &amp; Chọn Ảnh</v>
       </c>
-      <c r="C38" t="str">
+      <c r="C40" t="str">
         <v>Xác thực mã PIN khi truy cập Album ảnh riêng tư (/album/:id)</v>
       </c>
-      <c r="D38" t="str">
+      <c r="D40" t="str">
         <v>Khách hàng nhận được link album</v>
       </c>
-      <c r="E38" t="str" xml:space="preserve">
+      <c r="E40" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở link /album/:id
 2. Màn hình bảo mật yêu cầu nhập PIN mở khóa
 3. Nhập thử mã PIN sai -&gt; Báo lỗi
 4. Nhập đúng mã PIN -&gt; Bấm "Mở Album"</v>
       </c>
-      <c r="F38" t="str">
+      <c r="F40" t="str">
         <v>Nhập sai bị chặn; nhập đúng mở toàn bộ ảnh trong album kèm lời chào từ Studio.</v>
       </c>
-      <c r="G38" t="str">
-        <v>High</v>
-      </c>
-      <c r="H38" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I38" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J38" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="39" xml:space="preserve">
-      <c r="A39" t="str">
+      <c r="G40" t="str">
+        <v>High</v>
+      </c>
+      <c r="H40" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I40" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J40" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="41" xml:space="preserve">
+      <c r="A41" t="str">
         <v>TC_CLIENT_002</v>
       </c>
-      <c r="B39" t="str">
+      <c r="B41" t="str">
         <v>6. Khách Hàng Chọn Ảnh</v>
       </c>
-      <c r="C39" t="str">
+      <c r="C41" t="str">
         <v>Trải nghiệm xem ảnh toàn màn hình (Lightbox) trên Mobile &amp; PC</v>
       </c>
-      <c r="D39" t="str">
+      <c r="D41" t="str">
         <v>Đã mở khóa album</v>
       </c>
-      <c r="E39" t="str" xml:space="preserve">
+      <c r="E41" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm vào một bức ảnh để phóng to toàn màn hình
 2. Bấm phím mũi tên Trái/Phải hoặc vuốt trên màn hình cảm ứng
 3. Thử tính năng Phóng to (Zoom) &amp; Thu nhỏ</v>
       </c>
-      <c r="F39" t="str">
+      <c r="F41" t="str">
         <v>Xem ảnh nét căng, chuyển ảnh mượt mà, hỗ trợ tốt trên mọi kích thước màn hình.</v>
       </c>
-      <c r="G39" t="str">
-        <v>High</v>
-      </c>
-      <c r="H39" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I39" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J39" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="40" xml:space="preserve">
-      <c r="A40" t="str">
+      <c r="G41" t="str">
+        <v>High</v>
+      </c>
+      <c r="H41" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I41" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J41" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="42" xml:space="preserve">
+      <c r="A42" t="str">
         <v>TC_CLIENT_003</v>
       </c>
-      <c r="B40" t="str">
+      <c r="B42" t="str">
         <v>6. Khách Hàng Chọn Ảnh</v>
       </c>
-      <c r="C40" t="str">
+      <c r="C42" t="str">
         <v>Thao tác Thả tim / Chọn ảnh &amp; Bộ đếm giới hạn (Counter)</v>
       </c>
-      <c r="D40" t="str">
+      <c r="D42" t="str">
         <v>Album đang ở chế độ cho phép chọn ảnh</v>
       </c>
-      <c r="E40" t="str" xml:space="preserve">
+      <c r="E42" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm vào icon Trái tim trên ảnh để chọn ảnh ưng ý
 2. Theo dõi thanh tiến trình ở góc màn hình: "Đã chọn X / Y ảnh"
 3. Thử chọn vượt quá hạn mức tối đa cho phép</v>
       </c>
-      <c r="F40" t="str">
+      <c r="F42" t="str">
         <v>Thanh đếm cập nhật tức thì; nếu chọn vượt quá số lượng sẽ có cảnh báo nhắc nhở.</v>
       </c>
-      <c r="G40" t="str">
-        <v>High</v>
-      </c>
-      <c r="H40" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I40" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J40" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="41" xml:space="preserve">
-      <c r="A41" t="str">
+      <c r="G42" t="str">
+        <v>High</v>
+      </c>
+      <c r="H42" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I42" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J42" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="43" xml:space="preserve">
+      <c r="A43" t="str">
         <v>TC_CLIENT_004</v>
       </c>
-      <c r="B41" t="str">
+      <c r="B43" t="str">
         <v>6. Khách Hàng Chọn Ảnh</v>
       </c>
-      <c r="C41" t="str">
+      <c r="C43" t="str">
         <v>Nhập ghi chú chỉnh sửa &amp; Gửi danh sách chọn về Studio</v>
       </c>
-      <c r="D41" t="str">
+      <c r="D43" t="str">
         <v>Đã chọn đủ số lượng ảnh ưng ý</v>
       </c>
-      <c r="E41" t="str" xml:space="preserve">
+      <c r="E43" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút "Xem Các Ảnh Đã Chọn"
 2. Tại mỗi ảnh, nhập ghi chú chỉnh sửa (VD: "xóa vết bẩn trên áo, bóp eo nhẹ")
 3. Bấm nút "Gửi Danh Sách Ảnh Đã Chọn Cho Studio"
 4. Xác nhận gửi</v>
       </c>
-      <c r="F41" t="str">
+      <c r="F43" t="str">
         <v>Gửi thành công, khóa danh sách chọn (không thể đổi lại trừ khi Studio mở khóa), Studio nhận được danh sách ngay.</v>
       </c>
-      <c r="G41" t="str">
-        <v>High</v>
-      </c>
-      <c r="H41" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I41" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J41" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="42" xml:space="preserve">
-      <c r="A42" t="str">
+      <c r="G43" t="str">
+        <v>High</v>
+      </c>
+      <c r="H43" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I43" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J43" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="44" xml:space="preserve">
+      <c r="A44" t="str">
         <v>TC_CLIENT_005</v>
       </c>
-      <c r="B42" t="str">
+      <c r="B44" t="str">
         <v>6. Khách Hàng Chọn Ảnh</v>
       </c>
-      <c r="C42" t="str">
+      <c r="C44" t="str">
         <v>Tải ảnh chất lượng cao về máy (Single &amp; Batch Download)</v>
       </c>
-      <c r="D42" t="str">
+      <c r="D44" t="str">
         <v>Đã mở khóa album</v>
       </c>
-      <c r="E42" t="str" xml:space="preserve">
+      <c r="E44" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thử bấm nút Tải xuống trên từng tấm ảnh đơn lẻ
 2. Thử bấm nút "Tải Về Toàn Bộ Ảnh (File ZIP)"</v>
       </c>
-      <c r="F42" t="str">
+      <c r="F44" t="str">
         <v>Tải về ảnh gốc độ nét cao thành công, file zip chứa đầy đủ ảnh không bị lỗi.</v>
       </c>
-      <c r="G42" t="str">
+      <c r="G44" t="str">
         <v>Medium</v>
       </c>
-      <c r="H42" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I42" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J42" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="43" xml:space="preserve">
-      <c r="A43" t="str">
+      <c r="H44" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I44" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J44" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="45" xml:space="preserve">
+      <c r="A45" t="str">
         <v>TC_ADM_001</v>
       </c>
-      <c r="B43" t="str">
+      <c r="B45" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C43" t="str">
+      <c r="C45" t="str">
         <v>Đăng nhập trang Quản trị Master Admin tại /admin</v>
       </c>
-      <c r="D43" t="str">
+      <c r="D45" t="str">
         <v>Có tài khoản quản trị viên</v>
       </c>
-      <c r="E43" t="str" xml:space="preserve">
+      <c r="E45" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Truy cập /admin
 2. Đăng nhập bằng tài khoản master admin
 3. Quan sát Bảng điều khiển (Admin Dashboard)</v>
       </c>
-      <c r="F43" t="str">
+      <c r="F45" t="str">
         <v>Đăng nhập thành công, hiển thị các thẻ thống kê tổng số Người dùng, Nhiếp ảnh gia, Lịch chụp, Album và Cẩm nang.</v>
       </c>
-      <c r="G43" t="str">
-        <v>High</v>
-      </c>
-      <c r="H43" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I43" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J43" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="44" xml:space="preserve">
-      <c r="A44" t="str">
+      <c r="G45" t="str">
+        <v>High</v>
+      </c>
+      <c r="H45" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I45" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J45" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="46" xml:space="preserve">
+      <c r="A46" t="str">
         <v>TC_ADM_002</v>
       </c>
-      <c r="B44" t="str">
+      <c r="B46" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C44" t="str">
+      <c r="C46" t="str">
         <v>Quản trị Cẩm nang Địa điểm chụp (Thêm mới, Chỉnh sửa, Xóa)</v>
       </c>
-      <c r="D44" t="str">
+      <c r="D46" t="str">
         <v>Đang ở mục "Cẩm nang Địa điểm"</v>
       </c>
-      <c r="E44" t="str" xml:space="preserve">
+      <c r="E46" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm "Thêm Địa Điểm Mới"
 2. Nhập Tên địa điểm, chọn Tỉnh/Thành -&gt; chọn Phường/Xã -&gt; nhập Số nhà
 3. Nhập Giờ vàng, Giá vé, Mẹo góc máy, Concept, Link video review
@@ -1955,892 +2023,892 @@
 5. Bấm nút Sửa để thay đổi thông tin -&gt; Bấm Lưu
 6. Bấm nút Xóa để gỡ bỏ địa điểm</v>
       </c>
-      <c r="F44" t="str">
+      <c r="F46" t="str">
         <v>Các thao tác CRUD địa điểm hoạt động hoàn hảo, dữ liệu đồng bộ ngay lập tức lên Landing Page.</v>
       </c>
-      <c r="G44" t="str">
-        <v>High</v>
-      </c>
-      <c r="H44" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I44" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J44" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="45" xml:space="preserve">
-      <c r="A45" t="str">
+      <c r="G46" t="str">
+        <v>High</v>
+      </c>
+      <c r="H46" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I46" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J46" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="47" xml:space="preserve">
+      <c r="A47" t="str">
         <v>TC_ADM_003</v>
       </c>
-      <c r="B45" t="str">
+      <c r="B47" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C45" t="str">
+      <c r="C47" t="str">
         <v>Khôi phục 8 địa điểm kinh điển mặc định (Reset Locations)</v>
       </c>
-      <c r="D45" t="str">
+      <c r="D47" t="str">
         <v>Đang ở mục Cẩm nang Địa điểm</v>
       </c>
-      <c r="E45" t="str" xml:space="preserve">
+      <c r="E47" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút "Khôi Phục Mẫu Ban Đầu"
 2. Xác nhận khôi phục</v>
       </c>
-      <c r="F45" t="str">
+      <c r="F47" t="str">
         <v>Hệ thống tự động nạp lại chuẩn xác 8 địa điểm mẫu (Hồ Gươm, Tràng An, Sa Pa, Hội An, Huế, Cầu Đất, Ba Son, Phú Quốc) với đầy đủ Phường/Xã và Số nhà.</v>
       </c>
-      <c r="G45" t="str">
+      <c r="G47" t="str">
         <v>Medium</v>
       </c>
-      <c r="H45" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I45" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J45" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="46" xml:space="preserve">
-      <c r="A46" t="str">
+      <c r="H47" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I47" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J47" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="48" xml:space="preserve">
+      <c r="A48" t="str">
         <v>TC_ADM_004</v>
       </c>
-      <c r="B46" t="str">
+      <c r="B48" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C46" t="str">
+      <c r="C48" t="str">
         <v>Quản trị Nhiếp ảnh gia &amp; Gạt nút "Trải nghiệm Tự do" vs "Khóa kiểm duyệt"</v>
       </c>
-      <c r="D46" t="str">
+      <c r="D48" t="str">
         <v>Đang ở mục "Quản trị Nhiếp ảnh gia"</v>
       </c>
-      <c r="E46" t="str" xml:space="preserve">
+      <c r="E48" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Quan sát công tắc chuyển đổi chế độ kiểm duyệt
 2. Gạt sang "Khóa kiểm duyệt": Thử đăng ký thợ mới -&gt; Tài khoản ở trạng thái Chờ duyệt
 3. Tại bảng admin, bấm "Phê Duyệt &amp; Kích Hoạt" cho thợ đó
 4. Gạt sang "Trải nghiệm Tự do": Thợ mới đăng ký được vào thẳng hệ thống</v>
       </c>
-      <c r="F46" t="str">
+      <c r="F48" t="str">
         <v>Cơ chế đóng/mở kiểm duyệt linh hoạt, phê duyệt và khóa tài khoản tức thì.</v>
       </c>
-      <c r="G46" t="str">
-        <v>High</v>
-      </c>
-      <c r="H46" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I46" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J46" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="47" xml:space="preserve">
-      <c r="A47" t="str">
+      <c r="G48" t="str">
+        <v>High</v>
+      </c>
+      <c r="H48" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I48" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J48" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="49" xml:space="preserve">
+      <c r="A49" t="str">
         <v>TC_ADM_005</v>
       </c>
-      <c r="B47" t="str">
+      <c r="B49" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C47" t="str">
+      <c r="C49" t="str">
         <v>Quản trị Người dùng &amp; Xuất danh bạ CSV/Excel</v>
       </c>
-      <c r="D47" t="str">
+      <c r="D49" t="str">
         <v>Đang ở mục "Quản lý Người dùng"</v>
       </c>
-      <c r="E47" t="str" xml:space="preserve">
+      <c r="E49" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Xem bảng danh sách người dùng đầy đủ cột Họ tên, SĐT, Email, Vai trò, Địa chỉ
 2. Thay đổi vai trò (Client &lt;-&gt; Photographer &lt;-&gt; Admin) qua dropdown
 3. Tìm kiếm theo tên hoặc khu vực
 4. Bấm "Xuất CSV / Danh Bạ"</v>
       </c>
-      <c r="F47" t="str">
+      <c r="F49" t="str">
         <v>Cập nhật phân quyền ngay lập tức; tải về file CSV tiếng Việt chuẩn UTF-8 chứa đầy đủ thông tin danh bạ.</v>
       </c>
-      <c r="G47" t="str">
-        <v>High</v>
-      </c>
-      <c r="H47" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I47" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J47" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="48" xml:space="preserve">
-      <c r="A48" t="str">
+      <c r="G49" t="str">
+        <v>High</v>
+      </c>
+      <c r="H49" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I49" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J49" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="50" xml:space="preserve">
+      <c r="A50" t="str">
         <v>TC_ADM_006</v>
       </c>
-      <c r="B48" t="str">
+      <c r="B50" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C48" t="str">
+      <c r="C50" t="str">
         <v>Quản trị Đơn đặt lịch (Bookings Management)</v>
       </c>
-      <c r="D48" t="str">
+      <c r="D50" t="str">
         <v>Đang ở mục "Quản trị Đơn đặt lịch"</v>
       </c>
-      <c r="E48" t="str" xml:space="preserve">
+      <c r="E50" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Xem toàn bộ các đơn đặt lịch chụp trong hệ thống
 2. Cập nhật trạng thái đơn: Chờ xử lý -&gt; Đã xác nhận -&gt; Đã hoàn thành -&gt; Hủy đơn
 3. Lọc đơn theo ngày chụp hoặc theo thợ ảnh phụ trách</v>
       </c>
-      <c r="F48" t="str">
+      <c r="F50" t="str">
         <v>Quản lý đơn chụp thông suốt, cập nhật trạng thái chuẩn xác.</v>
       </c>
-      <c r="G48" t="str">
-        <v>High</v>
-      </c>
-      <c r="H48" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I48" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J48" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="49" xml:space="preserve">
-      <c r="A49" t="str">
+      <c r="G50" t="str">
+        <v>High</v>
+      </c>
+      <c r="H50" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I50" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J50" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="51" xml:space="preserve">
+      <c r="A51" t="str">
         <v>TC_ADM_007</v>
       </c>
-      <c r="B49" t="str">
+      <c r="B51" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C49" t="str">
+      <c r="C51" t="str">
         <v>Quản trị Danh mục chụp ảnh (Categories) &amp; Dịch vụ cộng thêm (Add-ons)</v>
       </c>
-      <c r="D49" t="str">
+      <c r="D51" t="str">
         <v>Đang ở mục Danh mục / Addons</v>
       </c>
-      <c r="E49" t="str" xml:space="preserve">
+      <c r="E51" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thêm một gói chụp mới (Tên, Giá khởi điểm, Icon, Mô tả)
 2. Thêm một dịch vụ cộng thêm mới (VD: Quay flycam +1.000.000đ)
 3. Chỉnh sửa đơn giá và xóa dịch vụ không còn áp dụng</v>
       </c>
-      <c r="F49" t="str">
+      <c r="F51" t="str">
         <v>Form đặt lịch trên toàn hệ thống tự động cập nhật bảng giá và gói dịch vụ mới.</v>
       </c>
-      <c r="G49" t="str">
-        <v>High</v>
-      </c>
-      <c r="H49" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I49" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J49" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="50" xml:space="preserve">
-      <c r="A50" t="str">
+      <c r="G51" t="str">
+        <v>High</v>
+      </c>
+      <c r="H51" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I51" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J51" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="52" xml:space="preserve">
+      <c r="A52" t="str">
         <v>TC_ADM_008</v>
       </c>
-      <c r="B50" t="str">
+      <c r="B52" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C50" t="str">
+      <c r="C52" t="str">
         <v>Cài đặt Cấu hình Email (SMTP) &amp; Kiểm tra gửi thư thử nghiệm</v>
       </c>
-      <c r="D50" t="str">
+      <c r="D52" t="str">
         <v>Đang ở mục "Cài đặt Email"</v>
       </c>
-      <c r="E50" t="str" xml:space="preserve">
+      <c r="E52" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Nhập thông số SMTP Server, Port, Email gửi, Mật khẩu ứng dụng
 2. Bấm "Lưu Cấu Hình"
 3. Bấm "Gửi Thư Thử Nghiệm" đến email cá nhân</v>
       </c>
-      <c r="F50" t="str">
+      <c r="F52" t="str">
         <v>Hệ thống gửi email test thành công, đảm bảo các thông báo đặt lịch tự động gửi qua email trơn tru.</v>
       </c>
-      <c r="G50" t="str">
+      <c r="G52" t="str">
         <v>Medium</v>
       </c>
-      <c r="H50" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I50" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J50" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="51" xml:space="preserve">
-      <c r="A51" t="str">
+      <c r="H52" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I52" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J52" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="53" xml:space="preserve">
+      <c r="A53" t="str">
         <v>TC_ADM_009</v>
       </c>
-      <c r="B51" t="str">
+      <c r="B53" t="str">
         <v>7. Bảng Quản Trị Hệ Thống (Admin)</v>
       </c>
-      <c r="C51" t="str">
+      <c r="C53" t="str">
         <v>Cài đặt Kênh liên hệ chung (Hotline, Zalo, Fanpage, Địa chỉ trụ sở)</v>
       </c>
-      <c r="D51" t="str">
+      <c r="D53" t="str">
         <v>Đang ở mục "Cài đặt Liên hệ"</v>
       </c>
-      <c r="E51" t="str" xml:space="preserve">
+      <c r="E53" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Cập nhật Hotline, Số Zalo hỗ trợ, Link Facebook Messenger
 2. Bấm Lưu
 3. Ra ngoài trang chủ kiểm tra các nút liên hệ nổi góc màn hình</v>
       </c>
-      <c r="F51" t="str">
+      <c r="F53" t="str">
         <v>Các nút gọi điện, chat Zalo, Messenger trên toàn bộ website tự động nhảy đúng thông tin mới.</v>
       </c>
-      <c r="G51" t="str">
+      <c r="G53" t="str">
         <v>Medium</v>
       </c>
-      <c r="H51" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I51" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J51" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="52" xml:space="preserve">
-      <c r="A52" t="str">
+      <c r="H53" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I53" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J53" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="54" xml:space="preserve">
+      <c r="A54" t="str">
         <v>TC_GEO_001</v>
       </c>
-      <c r="B52" t="str">
+      <c r="B54" t="str">
         <v>8. Địa Lý Hành Chính GHN</v>
       </c>
-      <c r="C52" t="str">
+      <c r="C54" t="str">
         <v>Tải danh mục 34 Tỉnh / Thành phố từ Database nội bộ</v>
       </c>
-      <c r="D52" t="str">
+      <c r="D54" t="str">
         <v>Gọi API /api/address/provinces hoặc mở bất kỳ form địa chỉ nào</v>
       </c>
-      <c r="E52" t="str" xml:space="preserve">
+      <c r="E54" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở ô chọn Tỉnh/Thành phố
 2. Kiểm tra danh sách hiển thị</v>
       </c>
-      <c r="F52" t="str">
+      <c r="F54" t="str">
         <v>Tải đầy đủ 34 tỉnh thành nội bộ (Hà Nội, TP. Hồ Chí Minh, Đà Nẵng, Huế, Ninh Bình, Sa Pa, Cầu Đất...). Tốc độ phản hồi tức thì &lt; 50ms, chi phí 0đ.</v>
       </c>
-      <c r="G52" t="str">
-        <v>High</v>
-      </c>
-      <c r="H52" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I52" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J52" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="53" xml:space="preserve">
-      <c r="A53" t="str">
+      <c r="G54" t="str">
+        <v>High</v>
+      </c>
+      <c r="H54" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I54" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J54" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="55" xml:space="preserve">
+      <c r="A55" t="str">
         <v>TC_GEO_002</v>
       </c>
-      <c r="B53" t="str">
+      <c r="B55" t="str">
         <v>8. Địa Lý Hành Chính GHN</v>
       </c>
-      <c r="C53" t="str">
+      <c r="C55" t="str">
         <v>Tải tự động danh sách Phường / Xã tương ứng theo Tỉnh đã chọn</v>
       </c>
-      <c r="D53" t="str">
+      <c r="D55" t="str">
         <v>Đã chọn 1 tỉnh cụ thể</v>
       </c>
-      <c r="E53" t="str" xml:space="preserve">
+      <c r="E55" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Chọn Tỉnh Hà Nội (provinceId: 1000000)
 2. Kiểm tra danh sách 126 Phường/Xã của Hà Nội
 3. Đổi sang Tỉnh TP. Hồ Chí Minh -&gt; Kiểm tra danh sách phường xã cập nhật lại theo TP.HCM</v>
       </c>
-      <c r="F53" t="str">
+      <c r="F55" t="str">
         <v>Dữ liệu phường/xã đổi ngay lập tức theo tỉnh thành đã chọn, không bị treo hay lẫn lộn giữa các tỉnh.</v>
       </c>
-      <c r="G53" t="str">
-        <v>High</v>
-      </c>
-      <c r="H53" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I53" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J53" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="54" xml:space="preserve">
-      <c r="A54" t="str">
+      <c r="G55" t="str">
+        <v>High</v>
+      </c>
+      <c r="H55" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I55" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J55" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="56" xml:space="preserve">
+      <c r="A56" t="str">
         <v>TC_GEO_003</v>
       </c>
-      <c r="B54" t="str">
+      <c r="B56" t="str">
         <v>8. Địa Lý Hành Chính GHN</v>
       </c>
-      <c r="C54" t="str">
+      <c r="C56" t="str">
         <v>Cơ chế dự phòng Offline Database (Local JSON Fallback)</v>
       </c>
-      <c r="D54" t="str">
+      <c r="D56" t="str">
         <v>Mất kết nối Internet hoặc MongoDB tạm ngắt kết nối</v>
       </c>
-      <c r="E54" t="str" xml:space="preserve">
+      <c r="E56" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Ngắt kết nối MongoDB Atlas hoặc chạy ở chế độ useLocalDB
 2. Thử truy cập bộ chọn Tỉnh thành và Phường xã</v>
       </c>
-      <c r="F54" t="str">
+      <c r="F56" t="str">
         <v>Hệ thống tự động chuyển sang đọc file server/data/ghn_address_data.json nội bộ, toàn bộ dropdown vẫn hoạt động bình thường.</v>
       </c>
-      <c r="G54" t="str">
-        <v>High</v>
-      </c>
-      <c r="H54" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I54" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J54" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="55" xml:space="preserve">
-      <c r="A55" t="str">
+      <c r="G56" t="str">
+        <v>High</v>
+      </c>
+      <c r="H56" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I56" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J56" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="57" xml:space="preserve">
+      <c r="A57" t="str">
         <v>TC_AI_001</v>
       </c>
-      <c r="B55" t="str">
+      <c r="B57" t="str">
         <v>9. Tối Ưu Tìm Kiếm AI (AI SEO)</v>
       </c>
-      <c r="C55" t="str">
+      <c r="C57" t="str">
         <v>Kiểm tra tệp robots.txt phân quyền cho AI Crawlers</v>
       </c>
-      <c r="D55" t="str">
+      <c r="D57" t="str">
         <v>Truy cập https://chiasehinhanhchup-jnvz.vercel.app/robots.txt</v>
       </c>
-      <c r="E55" t="str" xml:space="preserve">
+      <c r="E57" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở URL /robots.txt trên trình duyệt
 2. Kiểm tra các dòng User-agent</v>
       </c>
-      <c r="F55" t="str">
+      <c r="F57" t="str">
         <v>Mở quyền cho GPTBot, ChatGPT-User, OAI-SearchBot, ClaudeBot, PerplexityBot, Google-Extended, Applebot; khai báo link Sitemap và llms.txt.</v>
       </c>
-      <c r="G55" t="str">
-        <v>High</v>
-      </c>
-      <c r="H55" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I55" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J55" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="56" xml:space="preserve">
-      <c r="A56" t="str">
+      <c r="G57" t="str">
+        <v>High</v>
+      </c>
+      <c r="H57" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I57" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J57" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="58" xml:space="preserve">
+      <c r="A58" t="str">
         <v>TC_AI_002</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B58" t="str">
         <v>9. Tối Ưu Tìm Kiếm AI (AI SEO)</v>
       </c>
-      <c r="C56" t="str">
+      <c r="C58" t="str">
         <v>Kiểm tra tệp chuẩn ngữ cảnh LLM: /llms.txt</v>
       </c>
-      <c r="D56" t="str">
+      <c r="D58" t="str">
         <v>Truy cập https://chiasehinhanhchup-jnvz.vercel.app/llms.txt</v>
       </c>
-      <c r="E56" t="str" xml:space="preserve">
+      <c r="E58" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở URL /llms.txt trên trình duyệt
 2. Kiểm tra cấu trúc văn bản Markdown</v>
       </c>
-      <c r="F56" t="str">
+      <c r="F58" t="str">
         <v>Cung cấp bản tóm tắt tinh gọn về Photodate, dịch vụ chụp, cẩm nang tọa độ, link chính và cặp câu hỏi Q&amp;A chuẩn để AI trích dẫn.</v>
       </c>
-      <c r="G56" t="str">
-        <v>High</v>
-      </c>
-      <c r="H56" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I56" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J56" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="57" xml:space="preserve">
-      <c r="A57" t="str">
+      <c r="G58" t="str">
+        <v>High</v>
+      </c>
+      <c r="H58" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I58" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J58" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="59" xml:space="preserve">
+      <c r="A59" t="str">
         <v>TC_AI_003</v>
       </c>
-      <c r="B57" t="str">
+      <c r="B59" t="str">
         <v>9. Tối Ưu Tìm Kiếm AI (AI SEO)</v>
       </c>
-      <c r="C57" t="str">
+      <c r="C59" t="str">
         <v>Kiểm tra Sơ đồ trang web: /sitemap.xml</v>
       </c>
-      <c r="D57" t="str">
+      <c r="D59" t="str">
         <v>Truy cập https://chiasehinhanhchup-jnvz.vercel.app/sitemap.xml</v>
       </c>
-      <c r="E57" t="str" xml:space="preserve">
+      <c r="E59" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở URL /sitemap.xml trên trình duyệt
 2. Kiểm tra cú pháp XML chuẩn</v>
       </c>
-      <c r="F57" t="str">
+      <c r="F59" t="str">
         <v>Hiển thị cây thư mục liên kết hợp lệ, giúp bot tìm kiếm và bot AI lập chỉ mục toàn bộ các trang.</v>
       </c>
-      <c r="G57" t="str">
+      <c r="G59" t="str">
         <v>Medium</v>
       </c>
-      <c r="H57" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I57" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J57" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="58" xml:space="preserve">
-      <c r="A58" t="str">
+      <c r="H59" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I59" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J59" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="60" xml:space="preserve">
+      <c r="A60" t="str">
         <v>TC_AI_004</v>
       </c>
-      <c r="B58" t="str">
+      <c r="B60" t="str">
         <v>9. Tối Ưu Tìm Kiếm AI (AI SEO)</v>
       </c>
-      <c r="C58" t="str">
+      <c r="C60" t="str">
         <v>Kiểm tra Thẻ Dữ liệu cấu trúc Schema.org JSON-LD (WebSite, Org, TouristAttraction)</v>
       </c>
-      <c r="D58" t="str">
+      <c r="D60" t="str">
         <v>Xem nguồn trang (View Source) trang chủ</v>
       </c>
-      <c r="E58" t="str" xml:space="preserve">
+      <c r="E60" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Nhấn Ctrl + U xem mã nguồn trang chủ
 2. Tìm kiếm chuỗi "application/ld+json"
 3. Đọc các khối schema</v>
       </c>
-      <c r="F58" t="str">
+      <c r="F60" t="str">
         <v>Có đầy đủ Schema WebSite, Organization, ProfessionalService, và khối ItemList chứa các thực thể TouristAttraction kèm PostalAddress cho từng địa điểm chụp.</v>
       </c>
-      <c r="G58" t="str">
-        <v>High</v>
-      </c>
-      <c r="H58" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I58" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J58" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="59" xml:space="preserve">
-      <c r="A59" t="str">
+      <c r="G60" t="str">
+        <v>High</v>
+      </c>
+      <c r="H60" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I60" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J60" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="61" xml:space="preserve">
+      <c r="A61" t="str">
         <v>TC_AI_005</v>
       </c>
-      <c r="B59" t="str">
+      <c r="B61" t="str">
         <v>9. Tối Ưu Tìm Kiếm AI (AI SEO)</v>
       </c>
-      <c r="C59" t="str">
+      <c r="C61" t="str">
         <v>Kiểm tra Thẻ Open Graph &amp; Twitter Cards khi chia sẻ mạng xã hội</v>
       </c>
-      <c r="D59" t="str">
+      <c r="D61" t="str">
         <v>Chia sẻ link web lên Facebook / Zalo / Telegram</v>
       </c>
-      <c r="E59" t="str" xml:space="preserve">
+      <c r="E61" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Dán link web vào khung chat Zalo / Facebook
 2. Quan sát hình ảnh và tiêu đề xem trước</v>
       </c>
-      <c r="F59" t="str">
+      <c r="F61" t="str">
         <v>Hiển thị ảnh cover sắc nét, tiêu đề và mô tả chuyên nghiệp, không bị lỗi font.</v>
       </c>
-      <c r="G59" t="str">
+      <c r="G61" t="str">
         <v>Medium</v>
       </c>
-      <c r="H59" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I59" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J59" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="60" xml:space="preserve">
-      <c r="A60" t="str">
+      <c r="H61" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I61" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J61" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="62" xml:space="preserve">
+      <c r="A62" t="str">
         <v>TC_UI_001</v>
       </c>
-      <c r="B60" t="str">
+      <c r="B62" t="str">
         <v>10. Giao Diện &amp; Trải Nghiệm (UI/UX)</v>
       </c>
-      <c r="C60" t="str">
+      <c r="C62" t="str">
         <v>Chế độ Chống sập trang toàn cục (ErrorBoundary)</v>
       </c>
-      <c r="D60" t="str">
+      <c r="D62" t="str">
         <v>Trang web đang chạy</v>
       </c>
-      <c r="E60" t="str" xml:space="preserve">
+      <c r="E62" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Kiểm tra trong toàn bộ quá trình sử dụng nếu có lỗi JavaScript phát sinh đột ngột
 2. Quan sát màn hình hiển thị</v>
       </c>
-      <c r="F60" t="str">
+      <c r="F62" t="str">
         <v>Không bao giờ xuất hiện màn hình trắng bóc (blank screen); hiển thị giao diện báo sự cố thân thiện kèm nút "Tải lại trang" và "Về trang chủ".</v>
       </c>
-      <c r="G60" t="str">
-        <v>High</v>
-      </c>
-      <c r="H60" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I60" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J60" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="61" xml:space="preserve">
-      <c r="A61" t="str">
+      <c r="G62" t="str">
+        <v>High</v>
+      </c>
+      <c r="H62" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I62" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J62" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="63" xml:space="preserve">
+      <c r="A63" t="str">
         <v>TC_UI_002</v>
       </c>
-      <c r="B61" t="str">
+      <c r="B63" t="str">
         <v>10. Giao Diện &amp; Trải Nghiệm (UI/UX)</v>
       </c>
-      <c r="C61" t="str">
+      <c r="C63" t="str">
         <v>Chuyển đổi Chế độ Sáng / Tối (Dark / Light Theme)</v>
       </c>
-      <c r="D61" t="str">
+      <c r="D63" t="str">
         <v>Ở bất kỳ trang nào</v>
       </c>
-      <c r="E61" t="str" xml:space="preserve">
+      <c r="E63" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Bấm nút biểu tượng Mặt trời / Mặt trăng trên Header
 2. Quan sát màu nền, bảng biểu, thẻ card và phông chữ</v>
       </c>
-      <c r="F61" t="str">
+      <c r="F63" t="str">
         <v>Màu sắc đảo mượt mà, độ tương phản cao, giữ nguyên tính thẩm mỹ cao cấp của giao diện.</v>
       </c>
-      <c r="G61" t="str">
+      <c r="G63" t="str">
         <v>Medium</v>
       </c>
-      <c r="H61" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I61" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J61" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="62" xml:space="preserve">
-      <c r="A62" t="str">
+      <c r="H63" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I63" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J63" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="64" xml:space="preserve">
+      <c r="A64" t="str">
         <v>TC_UI_003</v>
       </c>
-      <c r="B62" t="str">
+      <c r="B64" t="str">
         <v>10. Giao Diện &amp; Trải Nghiệm (UI/UX)</v>
       </c>
-      <c r="C62" t="str">
+      <c r="C64" t="str">
         <v>Khả năng co giãn trên thiết bị di động (Mobile Responsive)</v>
       </c>
-      <c r="D62" t="str">
+      <c r="D64" t="str">
         <v>Mở web trên điện thoại iPhone / Android hoặc bật F12 Mobile View</v>
       </c>
-      <c r="E62" t="str" xml:space="preserve">
+      <c r="E64" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Kiểm tra Navbar thu gọn thành Menu Hamburger
 2. Kiểm tra các lưới ảnh và bảng biểu tự động xuống dòng phù hợp
 3. Thao tác vuốt chạm các nút bấm và popup</v>
       </c>
-      <c r="F62" t="str">
+      <c r="F64" t="str">
         <v>Giao diện không bị tràn viền ngang (no horizontal overflow), nút bấm to rõ dễ thao tác bằng ngón tay.</v>
       </c>
-      <c r="G62" t="str">
-        <v>High</v>
-      </c>
-      <c r="H62" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I62" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J62" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="63" xml:space="preserve">
-      <c r="A63" t="str">
+      <c r="G64" t="str">
+        <v>High</v>
+      </c>
+      <c r="H64" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I64" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J64" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="65" xml:space="preserve">
+      <c r="A65" t="str">
         <v>TC_UI_004</v>
       </c>
-      <c r="B63" t="str">
+      <c r="B65" t="str">
         <v>10. Giao Diện &amp; Trải Nghiệm (UI/UX)</v>
       </c>
-      <c r="C63" t="str">
+      <c r="C65" t="str">
         <v>Kiểm tra Cụm Nút Liên Hệ Nổi (Floating Contact Action Buttons)</v>
       </c>
-      <c r="D63" t="str">
+      <c r="D65" t="str">
         <v>Cuộn trang bất kỳ</v>
       </c>
-      <c r="E63" t="str" xml:space="preserve">
+      <c r="E65" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Quan sát góc dưới màn hình có cụm nút tròn: Hotline, Zalo, Messenger
 2. Lần lượt bấm vào từng nút</v>
       </c>
-      <c r="F63" t="str">
+      <c r="F65" t="str">
         <v>Các nút có hiệu ứng sóng rung thu hút, bấm vào liên kết chính xác đến số điện thoại và trang chat hỗ trợ.</v>
       </c>
-      <c r="G63" t="str">
+      <c r="G65" t="str">
         <v>Medium</v>
       </c>
-      <c r="H63" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I63" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J63" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="64" xml:space="preserve">
-      <c r="A64" t="str">
+      <c r="H65" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I65" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J65" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="66" xml:space="preserve">
+      <c r="A66" t="str">
         <v>TC_PERF_001</v>
       </c>
-      <c r="B64" t="str">
+      <c r="B66" t="str">
         <v>11. Hiệu Năng &amp; Tốc Độ</v>
       </c>
-      <c r="C64" t="str">
+      <c r="C66" t="str">
         <v>Tốc độ tải trang đầu tiên (First Contentful Paint)</v>
       </c>
-      <c r="D64" t="str">
+      <c r="D66" t="str">
         <v>Mở trang web trên trình duyệt sạch cache</v>
       </c>
-      <c r="E64" t="str" xml:space="preserve">
+      <c r="E66" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Tải trang chủ Photodate
 2. Đo thời gian hiển thị nội dung đầu tiên</v>
       </c>
-      <c r="F64" t="str">
+      <c r="F66" t="str">
         <v>Nội dung hiển thị &lt; 1.5 giây, tài nguyên CSS/JS được nén gzip và minify tối ưu.</v>
       </c>
-      <c r="G64" t="str">
-        <v>High</v>
-      </c>
-      <c r="H64" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I64" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J64" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="65" xml:space="preserve">
-      <c r="A65" t="str">
+      <c r="G66" t="str">
+        <v>High</v>
+      </c>
+      <c r="H66" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I66" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J66" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="67" xml:space="preserve">
+      <c r="A67" t="str">
         <v>TC_PERF_002</v>
       </c>
-      <c r="B65" t="str">
+      <c r="B67" t="str">
         <v>11. Hiệu Năng &amp; Tốc Độ</v>
       </c>
-      <c r="C65" t="str">
+      <c r="C67" t="str">
         <v>Tải chậm hình ảnh thông minh (Lazy Loading Images)</v>
       </c>
-      <c r="D65" t="str">
+      <c r="D67" t="str">
         <v>Ở trang chủ có nhiều ảnh cẩm nang và portfolio</v>
       </c>
-      <c r="E65" t="str" xml:space="preserve">
+      <c r="E67" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Mở tab Network trong DevTools
 2. Cuộn từ từ xuống các khối dưới cùng của trang</v>
       </c>
-      <c r="F65" t="str">
+      <c r="F67" t="str">
         <v>Ảnh chỉ được tải khi người dùng cuộn đến gần màn hình nhìn thấy, tiết kiệm băng thông tối đa.</v>
       </c>
-      <c r="G65" t="str">
+      <c r="G67" t="str">
         <v>Medium</v>
       </c>
-      <c r="H65" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I65" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J65" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="66" xml:space="preserve">
-      <c r="A66" t="str">
+      <c r="H67" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I67" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J67" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="68" xml:space="preserve">
+      <c r="A68" t="str">
         <v>TC_PERF_003</v>
       </c>
-      <c r="B66" t="str">
+      <c r="B68" t="str">
         <v>11. Hiệu Năng &amp; Tốc Độ</v>
       </c>
-      <c r="C66" t="str">
+      <c r="C68" t="str">
         <v>Tối ưu hóa bộ nhớ khi xem hàng trăm ảnh trong Album (Virtualization/Pagination)</v>
       </c>
-      <c r="D66" t="str">
+      <c r="D68" t="str">
         <v>Mở album có &gt; 200 ảnh</v>
       </c>
-      <c r="E66" t="str" xml:space="preserve">
+      <c r="E68" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Cuộn xem toàn bộ album ảnh
 2. Quan sát độ mượt của trình duyệt</v>
       </c>
-      <c r="F66" t="str">
+      <c r="F68" t="str">
         <v>Trình duyệt không bị giật lag hay quá tải bộ nhớ RAM.</v>
       </c>
-      <c r="G66" t="str">
-        <v>High</v>
-      </c>
-      <c r="H66" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I66" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J66" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="str">
+      <c r="G68" t="str">
+        <v>High</v>
+      </c>
+      <c r="H68" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I68" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J68" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="str">
         <v>TC_SEC_001</v>
-      </c>
-      <c r="B67" t="str">
-        <v>12. Bảo Mật &amp; An Toàn</v>
-      </c>
-      <c r="C67" t="str">
-        <v>Bảo mật mật khẩu người dùng (Hashing Password)</v>
-      </c>
-      <c r="D67" t="str">
-        <v>Kiểm tra cơ sở dữ liệu backend</v>
-      </c>
-      <c r="E67" t="str">
-        <v>1. Xem trực tiếp bản ghi User trong DB</v>
-      </c>
-      <c r="F67" t="str">
-        <v>Mật khẩu phải được mã hóa bằng thuật toán băm an toàn (bcrypt/hash), tuyệt đối không lưu dạng plain text.</v>
-      </c>
-      <c r="G67" t="str">
-        <v>High</v>
-      </c>
-      <c r="H67" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I67" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J67" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="str">
-        <v>TC_SEC_002</v>
-      </c>
-      <c r="B68" t="str">
-        <v>12. Bảo Mật &amp; An Toàn</v>
-      </c>
-      <c r="C68" t="str">
-        <v>Bảo mật quyền truy cập Album qua mã PIN</v>
-      </c>
-      <c r="D68" t="str">
-        <v>Album có thiết lập mã PIN</v>
-      </c>
-      <c r="E68" t="str">
-        <v>1. Gọi trực tiếp API lấy ảnh của album mà không truyền mã PIN hoặc truyền sai PIN</v>
-      </c>
-      <c r="F68" t="str">
-        <v>Backend trả về mã lỗi 401/403 Unauthorized, không trả về link ảnh gốc.</v>
-      </c>
-      <c r="G68" t="str">
-        <v>High</v>
-      </c>
-      <c r="H68" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I68" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J68" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="69" xml:space="preserve">
-      <c r="A69" t="str">
-        <v>TC_SEC_003</v>
       </c>
       <c r="B69" t="str">
         <v>12. Bảo Mật &amp; An Toàn</v>
       </c>
       <c r="C69" t="str">
+        <v>Bảo mật mật khẩu người dùng (Hashing Password)</v>
+      </c>
+      <c r="D69" t="str">
+        <v>Kiểm tra cơ sở dữ liệu backend</v>
+      </c>
+      <c r="E69" t="str">
+        <v>1. Xem trực tiếp bản ghi User trong DB</v>
+      </c>
+      <c r="F69" t="str">
+        <v>Mật khẩu phải được mã hóa bằng thuật toán băm an toàn (bcrypt/hash), tuyệt đối không lưu dạng plain text.</v>
+      </c>
+      <c r="G69" t="str">
+        <v>High</v>
+      </c>
+      <c r="H69" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I69" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J69" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="str">
+        <v>TC_SEC_002</v>
+      </c>
+      <c r="B70" t="str">
+        <v>12. Bảo Mật &amp; An Toàn</v>
+      </c>
+      <c r="C70" t="str">
+        <v>Bảo mật quyền truy cập Album qua mã PIN</v>
+      </c>
+      <c r="D70" t="str">
+        <v>Album có thiết lập mã PIN</v>
+      </c>
+      <c r="E70" t="str">
+        <v>1. Gọi trực tiếp API lấy ảnh của album mà không truyền mã PIN hoặc truyền sai PIN</v>
+      </c>
+      <c r="F70" t="str">
+        <v>Backend trả về mã lỗi 401/403 Unauthorized, không trả về link ảnh gốc.</v>
+      </c>
+      <c r="G70" t="str">
+        <v>High</v>
+      </c>
+      <c r="H70" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I70" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J70" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="71" xml:space="preserve">
+      <c r="A71" t="str">
+        <v>TC_SEC_003</v>
+      </c>
+      <c r="B71" t="str">
+        <v>12. Bảo Mật &amp; An Toàn</v>
+      </c>
+      <c r="C71" t="str">
         <v>Chống tấn công XSS trong trường Bio, Mô tả &amp; Ghi chú</v>
       </c>
-      <c r="D69" t="str">
+      <c r="D71" t="str">
         <v>Form nhập liệu (Bio, Ghi chú cẩm nang, Ghi chú đặt lịch)</v>
       </c>
-      <c r="E69" t="str" xml:space="preserve">
+      <c r="E71" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thử nhập đoạn mã độc: &lt;script&gt;alert("XSS")&lt;/script&gt;
 2. Lưu và xem lại nội dung hiển thị</v>
       </c>
-      <c r="F69" t="str">
+      <c r="F71" t="str">
         <v>Đoạn mã được chuyển đổi thành chuỗi text an toàn hoặc bị lọc bỏ, không thực thi mã độc trên trình duyệt.</v>
       </c>
-      <c r="G69" t="str">
-        <v>High</v>
-      </c>
-      <c r="H69" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I69" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J69" t="str">
-        <v>Đã kiểm tra trên bản 2.0</v>
-      </c>
-    </row>
-    <row r="70" xml:space="preserve">
-      <c r="A70" t="str">
+      <c r="G71" t="str">
+        <v>High</v>
+      </c>
+      <c r="H71" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I71" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J71" t="str">
+        <v>Đã kiểm tra trên bản 2.0</v>
+      </c>
+    </row>
+    <row r="72" xml:space="preserve">
+      <c r="A72" t="str">
         <v>TC_SEC_004</v>
       </c>
-      <c r="B70" t="str">
+      <c r="B72" t="str">
         <v>12. Bảo Mật &amp; An Toàn</v>
       </c>
-      <c r="C70" t="str">
+      <c r="C72" t="str">
         <v>Giới hạn kích thước file tải lên (Upload Limit &amp; Type Check)</v>
       </c>
-      <c r="D70" t="str">
+      <c r="D72" t="str">
         <v>Form tải ảnh lên album hoặc avatar</v>
       </c>
-      <c r="E70" t="str" xml:space="preserve">
+      <c r="E72" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Thử tải file không phải ảnh (.exe, .pdf, .bat)
 2. Thử tải file ảnh dung lượng quá lớn vượt quy định</v>
       </c>
-      <c r="F70" t="str">
+      <c r="F72" t="str">
         <v>Hệ thống từ chối file không đúng định dạng và báo lỗi dung lượng vượt mức.</v>
       </c>
-      <c r="G70" t="str">
-        <v>High</v>
-      </c>
-      <c r="H70" t="str">
-        <v>Pass</v>
-      </c>
-      <c r="I70" t="str">
-        <v>Tester / QA Lead</v>
-      </c>
-      <c r="J70" t="str">
+      <c r="G72" t="str">
+        <v>High</v>
+      </c>
+      <c r="H72" t="str">
+        <v>Pass</v>
+      </c>
+      <c r="I72" t="str">
+        <v>Tester / QA Lead</v>
+      </c>
+      <c r="J72" t="str">
         <v>Đã kiểm tra trên bản 2.0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J70"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J72"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>